<commit_message>
adjust paper size margin etc for PO template
</commit_message>
<xml_diff>
--- a/po_template/PO TH TEMPLATE.xlsx
+++ b/po_template/PO TH TEMPLATE.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EVERBEST\NEW_GENERATOR\webapp\po_template\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93591AF1-C305-438A-A00F-2277F9FA4AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7500"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -386,17 +392,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="7">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="[$-409]d\-mmm\-yy;@"/>
-    <numFmt numFmtId="179" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="[$-409]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
-  <fonts count="50">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -560,150 +564,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -734,8 +594,15 @@
       <name val="SimSun"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="38">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -778,188 +645,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="54">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -1508,463 +1195,389 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="51">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="46" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="47" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="47" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="48" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="9" borderId="49" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="50" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="49" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="11" borderId="51" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="52" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="53" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="31" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="58" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="58" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="11" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="4" fontId="11" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="15" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="5" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="11" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="12" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="14" fillId="4" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="15" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="15" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="16" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="17" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1972,350 +1585,247 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="15" fillId="5" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="15" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="14" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="14" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="14" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="14" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="14" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="51">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 2" xfId="49"/>
-    <cellStyle name="Normal_Book1" xfId="50"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="Normal_Book1" xfId="4" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -2326,7 +1836,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -2354,161 +1864,47 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
@@ -2524,13 +1920,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="64" name="Picture 10"/>
+        <xdr:cNvPr id="64" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000040000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2566,13 +1968,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="65" name="Picture 12"/>
+        <xdr:cNvPr id="65" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000041000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2601,9 +2009,15 @@
       <xdr:rowOff>33020</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2734310" cy="464820"/>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="66" name="TextBox 4"/>
+        <xdr:cNvPr id="66" name="TextBox 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000042000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -2816,9 +2230,15 @@
       <xdr:row>21</xdr:row>
       <xdr:rowOff>338455</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Oval 12"/>
+        <xdr:cNvPr id="2" name="Oval 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -2973,13 +2393,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 4" descr="Tracce logo"/>
+        <xdr:cNvPr id="3" name="Picture 4" descr="Tracce logo">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3013,9 +2439,15 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>99060</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="AutoShape 54"/>
+        <xdr:cNvPr id="4" name="AutoShape 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks noChangeArrowheads="1"/>
         </xdr:cNvSpPr>
@@ -3188,13 +2620,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 2"/>
+        <xdr:cNvPr id="8" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3230,13 +2668,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Picture 4"/>
+        <xdr:cNvPr id="9" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3272,13 +2716,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Picture 13"/>
+        <xdr:cNvPr id="10" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3312,9 +2762,15 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>362902</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Oval 10"/>
+        <xdr:cNvPr id="11" name="Oval 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -3469,13 +2925,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Picture 13" descr="WhatsApp Image 2026-10-05 at 11.28.13 (1)"/>
+        <xdr:cNvPr id="14" name="Picture 13" descr="WhatsApp Image 2026-10-05 at 11.28.13 (1)">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
         <a:srcRect t="20457" r="454" b="13257"/>
         <a:stretch>
           <a:fillRect/>
@@ -3508,13 +2970,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Picture 14" descr="WhatsApp Image 2026-10-05 at 11.28.13"/>
+        <xdr:cNvPr id="15" name="Picture 14" descr="WhatsApp Image 2026-10-05 at 11.28.13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
         <a:srcRect l="27140" t="-1900" r="20474"/>
         <a:stretch>
           <a:fillRect/>
@@ -3779,668 +3247,670 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H53"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="8" width="40.7809523809524" customWidth="1"/>
+    <col min="1" max="8" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:8">
+    <row r="1" spans="1:8" ht="24.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="5" t="s">
+      <c r="E1" s="2"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1" spans="1:8">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="145" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="9" t="s">
+      <c r="C2" s="146"/>
+      <c r="E2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1" spans="1:8">
-      <c r="A3" s="11"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="14"/>
-      <c r="G3" s="15" t="s">
+    <row r="3" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A3" s="8"/>
+      <c r="B3" s="147"/>
+      <c r="C3" s="148"/>
+      <c r="E3" s="9"/>
+      <c r="G3" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="25" customHeight="1" spans="1:8">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="145" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="14"/>
-      <c r="G4" s="16" t="s">
+      <c r="C4" s="146"/>
+      <c r="E4" s="9"/>
+      <c r="G4" s="11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="25" customHeight="1" spans="1:8">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="149" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="18"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="14"/>
-      <c r="G5" s="16" t="s">
+      <c r="C5" s="150"/>
+      <c r="E5" s="9"/>
+      <c r="G5" s="11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" ht="25" customHeight="1" spans="1:8">
-      <c r="A6" s="19"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-    </row>
-    <row r="7" ht="25" customHeight="1" spans="1:8">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-    </row>
-    <row r="8" ht="30" customHeight="1" spans="1:8">
-      <c r="A8" s="24" t="s">
+    <row r="6" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A6" s="12"/>
+      <c r="B6" s="151"/>
+      <c r="C6" s="152"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" ht="30" customHeight="1">
+      <c r="A8" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="108" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="87" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="92" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="G8" s="94" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" spans="1:8">
-      <c r="A9" s="30"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="35"/>
-    </row>
-    <row r="10" ht="30" customHeight="1" spans="1:8">
-      <c r="A10" s="36"/>
-      <c r="B10" s="37" t="s">
+    <row r="9" spans="1:8" ht="30" customHeight="1">
+      <c r="A9" s="104"/>
+      <c r="B9" s="109"/>
+      <c r="C9" s="109"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="91"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="95"/>
+    </row>
+    <row r="10" spans="1:8" ht="30" customHeight="1">
+      <c r="A10" s="105"/>
+      <c r="B10" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="38"/>
-      <c r="E10" s="39" t="s">
+      <c r="D10" s="89"/>
+      <c r="E10" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="40" t="s">
+      <c r="F10" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="41" t="s">
+      <c r="G10" s="19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" spans="1:8">
-      <c r="A11" s="42"/>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="46">
+    <row r="11" spans="1:8" ht="30" customHeight="1">
+      <c r="A11" s="106"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="22">
         <v>0</v>
       </c>
-      <c r="G11" s="47">
+      <c r="G11" s="23">
         <f t="shared" ref="G11:G14" si="0">F11*E11</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1" spans="1:8">
-      <c r="A12" s="48"/>
-      <c r="B12" s="49"/>
-      <c r="C12" s="50"/>
-      <c r="D12" s="51"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="46">
+    <row r="12" spans="1:8" ht="30" customHeight="1">
+      <c r="A12" s="107"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="22">
         <v>0</v>
       </c>
-      <c r="G12" s="53">
+      <c r="G12" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1" spans="1:8">
-      <c r="A13" s="54" t="s">
+    <row r="13" spans="1:8" ht="30" customHeight="1">
+      <c r="A13" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="50"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="52"/>
-      <c r="F13" s="46">
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="22">
         <v>0</v>
       </c>
-      <c r="G13" s="53">
+      <c r="G13" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1" spans="1:8">
-      <c r="A14" s="55" t="s">
+    <row r="14" spans="1:8" ht="30" customHeight="1">
+      <c r="A14" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="56"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="46">
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="22">
         <v>0</v>
       </c>
-      <c r="G14" s="53">
+      <c r="G14" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" spans="1:8">
-      <c r="A15" s="58"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="59"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="60">
+    <row r="15" spans="1:8" ht="30" customHeight="1">
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="34">
         <f>SUM(E11:E14)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="61"/>
-      <c r="G15" s="62">
+      <c r="F15" s="35"/>
+      <c r="G15" s="36">
         <f>SUM(G11:G14)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="63"/>
-    </row>
-    <row r="16" ht="25" customHeight="1" spans="1:8">
-      <c r="A16" s="58"/>
-      <c r="B16" s="58"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="58"/>
-      <c r="G16" s="58"/>
-      <c r="H16" s="58"/>
-    </row>
-    <row r="17" ht="30" customHeight="1" spans="1:8">
-      <c r="A17" s="64" t="s">
+      <c r="H15" s="10"/>
+    </row>
+    <row r="16" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+    </row>
+    <row r="17" spans="1:8" ht="30" customHeight="1">
+      <c r="A17" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="65"/>
-      <c r="C17" s="66"/>
-      <c r="D17" s="67" t="s">
+      <c r="B17" s="96"/>
+      <c r="C17" s="97"/>
+      <c r="D17" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="68" t="s">
+      <c r="E17" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="F17" s="69" t="s">
+      <c r="F17" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="70"/>
-    </row>
-    <row r="18" ht="30" customHeight="1" spans="1:8">
-      <c r="A18" s="71" t="s">
+      <c r="G17" s="124"/>
+    </row>
+    <row r="18" spans="1:8" ht="30" customHeight="1">
+      <c r="A18" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="72"/>
-      <c r="C18" s="73"/>
-      <c r="D18" s="74"/>
-      <c r="E18" s="75"/>
-      <c r="F18" s="75"/>
-      <c r="G18" s="76"/>
-    </row>
-    <row r="19" ht="30" customHeight="1" spans="1:8">
-      <c r="A19" s="77" t="s">
+      <c r="B18" s="98"/>
+      <c r="C18" s="99"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="43"/>
+    </row>
+    <row r="19" spans="1:8" ht="30" customHeight="1">
+      <c r="A19" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="78"/>
-      <c r="C19" s="79"/>
-      <c r="D19" s="74"/>
-      <c r="E19" s="74"/>
-      <c r="F19" s="74"/>
-      <c r="G19" s="80"/>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:8">
-      <c r="A20" s="81" t="s">
+      <c r="B19" s="45"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="47"/>
+    </row>
+    <row r="20" spans="1:8" ht="30" customHeight="1">
+      <c r="A20" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="82"/>
-      <c r="C20" s="83"/>
-      <c r="D20" s="74"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="74"/>
-      <c r="G20" s="80"/>
-    </row>
-    <row r="21" ht="30" customHeight="1" spans="1:8">
-      <c r="A21" s="84" t="s">
+      <c r="B20" s="49"/>
+      <c r="C20" s="50"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="47"/>
+    </row>
+    <row r="21" spans="1:8" ht="30" customHeight="1">
+      <c r="A21" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="85" t="s">
+      <c r="B21" s="110" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="86"/>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="80"/>
-    </row>
-    <row r="22" ht="30" customHeight="1" spans="1:8">
-      <c r="A22" s="87"/>
-      <c r="B22" s="88"/>
-      <c r="C22" s="89"/>
-      <c r="D22" s="74"/>
-      <c r="E22" s="74"/>
-      <c r="F22" s="74"/>
-      <c r="G22" s="80"/>
-    </row>
-    <row r="23" ht="30" customHeight="1" spans="1:8">
-      <c r="A23" s="90" t="s">
+      <c r="C21" s="111"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="47"/>
+    </row>
+    <row r="22" spans="1:8" ht="30" customHeight="1">
+      <c r="A22" s="52"/>
+      <c r="B22" s="112"/>
+      <c r="C22" s="113"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="47"/>
+    </row>
+    <row r="23" spans="1:8" ht="30" customHeight="1">
+      <c r="A23" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="78"/>
-      <c r="C23" s="79"/>
-      <c r="D23" s="74"/>
-      <c r="E23" s="74"/>
-      <c r="F23" s="74"/>
-      <c r="G23" s="80"/>
-    </row>
-    <row r="24" ht="30" customHeight="1" spans="1:8">
-      <c r="A24" s="90" t="s">
+      <c r="B23" s="45"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="47"/>
+    </row>
+    <row r="24" spans="1:8" ht="30" customHeight="1">
+      <c r="A24" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="91"/>
-      <c r="C24" s="92"/>
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="74"/>
-      <c r="G24" s="80"/>
-    </row>
-    <row r="25" ht="30" customHeight="1" spans="1:8">
-      <c r="A25" s="93"/>
-      <c r="B25" s="94"/>
-      <c r="C25" s="95"/>
-      <c r="D25" s="96"/>
-      <c r="E25" s="96"/>
-      <c r="F25" s="96"/>
-      <c r="G25" s="97"/>
-    </row>
-    <row r="26" ht="25" customHeight="1" spans="1:8">
-      <c r="A26" s="98"/>
-      <c r="B26" s="98"/>
-      <c r="C26" s="99"/>
-      <c r="D26" s="99"/>
-      <c r="E26" s="100"/>
-      <c r="F26" s="58"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="58"/>
-    </row>
-    <row r="27" ht="25" customHeight="1" spans="1:8">
-      <c r="A27" s="101" t="s">
+      <c r="B24" s="53"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="47"/>
+    </row>
+    <row r="25" spans="1:8" ht="30" customHeight="1">
+      <c r="A25" s="55"/>
+      <c r="B25" s="56"/>
+      <c r="C25" s="57"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="58"/>
+      <c r="G25" s="59"/>
+    </row>
+    <row r="26" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A26" s="60"/>
+      <c r="B26" s="60"/>
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+    </row>
+    <row r="27" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A27" s="125" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="102"/>
-      <c r="C27" s="102"/>
-      <c r="D27" s="102"/>
-      <c r="E27" s="102"/>
-      <c r="F27" s="102"/>
-      <c r="G27" s="102"/>
-      <c r="H27" s="103"/>
-    </row>
-    <row r="28" ht="25" customHeight="1" spans="1:8">
-      <c r="A28" s="104">
+      <c r="B27" s="126"/>
+      <c r="C27" s="126"/>
+      <c r="D27" s="126"/>
+      <c r="E27" s="126"/>
+      <c r="F27" s="126"/>
+      <c r="G27" s="126"/>
+      <c r="H27" s="127"/>
+    </row>
+    <row r="28" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A28" s="128">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="B28" s="105"/>
-      <c r="C28" s="105"/>
-      <c r="D28" s="105"/>
-      <c r="E28" s="105"/>
-      <c r="F28" s="105"/>
-      <c r="G28" s="105"/>
-      <c r="H28" s="106"/>
-    </row>
-    <row r="29" ht="25" customHeight="1" spans="1:8">
-      <c r="A29" s="104">
+      <c r="B28" s="129"/>
+      <c r="C28" s="129"/>
+      <c r="D28" s="129"/>
+      <c r="E28" s="129"/>
+      <c r="F28" s="129"/>
+      <c r="G28" s="129"/>
+      <c r="H28" s="130"/>
+    </row>
+    <row r="29" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A29" s="128">
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="B29" s="105"/>
-      <c r="C29" s="105"/>
-      <c r="D29" s="105"/>
-      <c r="E29" s="105"/>
-      <c r="F29" s="105"/>
-      <c r="G29" s="105"/>
-      <c r="H29" s="106"/>
-    </row>
-    <row r="30" ht="25" customHeight="1" spans="1:8">
-      <c r="A30" s="107"/>
-      <c r="B30" s="108"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="109"/>
-      <c r="E30" s="110"/>
-      <c r="F30" s="111"/>
-      <c r="G30" s="110"/>
-      <c r="H30" s="112"/>
-    </row>
-    <row r="31" ht="25" customHeight="1" spans="1:8">
-      <c r="A31" s="113"/>
-      <c r="B31" s="114"/>
-      <c r="C31" s="113"/>
-      <c r="D31" s="115"/>
-      <c r="E31" s="116"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="116"/>
-      <c r="H31" s="117"/>
-    </row>
-    <row r="32" ht="25" customHeight="1" spans="1:8">
-      <c r="A32" s="113"/>
-      <c r="B32" s="114"/>
-      <c r="C32" s="113"/>
-      <c r="D32" s="115"/>
-      <c r="E32" s="116"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="116"/>
-      <c r="H32" s="117"/>
-    </row>
-    <row r="33" ht="25" customHeight="1" spans="1:8">
-      <c r="A33" s="113"/>
-      <c r="B33" s="114"/>
-      <c r="C33" s="113"/>
-      <c r="D33" s="115"/>
-      <c r="E33" s="116"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="116"/>
-      <c r="H33" s="117"/>
-    </row>
-    <row r="34" ht="25" customHeight="1" spans="1:8">
-      <c r="A34" s="113"/>
-      <c r="B34" s="114"/>
-      <c r="C34" s="113"/>
-      <c r="D34" s="115"/>
-      <c r="E34" s="116"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="116"/>
-      <c r="H34" s="117"/>
-    </row>
-    <row r="35" ht="25" customHeight="1" spans="1:8">
-      <c r="A35" s="113"/>
-      <c r="B35" s="114"/>
-      <c r="C35" s="113"/>
-      <c r="D35" s="115"/>
-      <c r="E35" s="116"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="116"/>
-      <c r="H35" s="117"/>
-    </row>
-    <row r="36" ht="25" customHeight="1" spans="1:8">
-      <c r="A36" s="113"/>
-      <c r="B36" s="114"/>
-      <c r="C36" s="113"/>
-      <c r="D36" s="115"/>
-      <c r="E36" s="116"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="116"/>
-      <c r="H36" s="117"/>
-    </row>
-    <row r="37" ht="25" customHeight="1" spans="1:8">
+      <c r="B29" s="129"/>
+      <c r="C29" s="129"/>
+      <c r="D29" s="129"/>
+      <c r="E29" s="129"/>
+      <c r="F29" s="129"/>
+      <c r="G29" s="129"/>
+      <c r="H29" s="130"/>
+    </row>
+    <row r="30" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A30" s="114"/>
+      <c r="B30" s="115"/>
+      <c r="C30" s="114"/>
+      <c r="D30" s="120"/>
+      <c r="E30" s="136"/>
+      <c r="F30" s="137"/>
+      <c r="G30" s="136"/>
+      <c r="H30" s="142"/>
+    </row>
+    <row r="31" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A31" s="116"/>
+      <c r="B31" s="117"/>
+      <c r="C31" s="116"/>
+      <c r="D31" s="121"/>
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="138"/>
+      <c r="H31" s="143"/>
+    </row>
+    <row r="32" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A32" s="116"/>
+      <c r="B32" s="117"/>
+      <c r="C32" s="116"/>
+      <c r="D32" s="121"/>
+      <c r="E32" s="138"/>
+      <c r="F32" s="139"/>
+      <c r="G32" s="138"/>
+      <c r="H32" s="143"/>
+    </row>
+    <row r="33" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A33" s="116"/>
+      <c r="B33" s="117"/>
+      <c r="C33" s="116"/>
+      <c r="D33" s="121"/>
+      <c r="E33" s="138"/>
+      <c r="F33" s="139"/>
+      <c r="G33" s="138"/>
+      <c r="H33" s="143"/>
+    </row>
+    <row r="34" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A34" s="116"/>
+      <c r="B34" s="117"/>
+      <c r="C34" s="116"/>
+      <c r="D34" s="121"/>
+      <c r="E34" s="138"/>
+      <c r="F34" s="139"/>
+      <c r="G34" s="138"/>
+      <c r="H34" s="143"/>
+    </row>
+    <row r="35" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A35" s="116"/>
+      <c r="B35" s="117"/>
+      <c r="C35" s="116"/>
+      <c r="D35" s="121"/>
+      <c r="E35" s="138"/>
+      <c r="F35" s="139"/>
+      <c r="G35" s="138"/>
+      <c r="H35" s="143"/>
+    </row>
+    <row r="36" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A36" s="116"/>
+      <c r="B36" s="117"/>
+      <c r="C36" s="116"/>
+      <c r="D36" s="121"/>
+      <c r="E36" s="138"/>
+      <c r="F36" s="139"/>
+      <c r="G36" s="138"/>
+      <c r="H36" s="143"/>
+    </row>
+    <row r="37" spans="1:8" ht="24.95" customHeight="1">
       <c r="A37" s="118"/>
       <c r="B37" s="119"/>
       <c r="C37" s="118"/>
-      <c r="D37" s="120"/>
-      <c r="E37" s="121"/>
-      <c r="F37" s="122"/>
-      <c r="G37" s="121"/>
-      <c r="H37" s="123"/>
-    </row>
-    <row r="38" ht="25" customHeight="1" spans="1:8">
-      <c r="A38" s="124">
+      <c r="D37" s="122"/>
+      <c r="E37" s="140"/>
+      <c r="F37" s="141"/>
+      <c r="G37" s="140"/>
+      <c r="H37" s="144"/>
+    </row>
+    <row r="38" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A38" s="131">
         <f>D11</f>
         <v>0</v>
       </c>
-      <c r="B38" s="125"/>
-      <c r="C38" s="126">
+      <c r="B38" s="132"/>
+      <c r="C38" s="133">
         <f>D12</f>
         <v>0</v>
       </c>
-      <c r="D38" s="127"/>
-      <c r="E38" s="126">
+      <c r="D38" s="134"/>
+      <c r="E38" s="133">
         <f>D13</f>
         <v>0</v>
       </c>
-      <c r="F38" s="128"/>
-      <c r="G38" s="126">
+      <c r="F38" s="135"/>
+      <c r="G38" s="133">
         <f>D14</f>
         <v>0</v>
       </c>
-      <c r="H38" s="128"/>
-    </row>
-    <row r="39" ht="25" customHeight="1" spans="1:8">
-      <c r="A39" s="129" t="s">
+      <c r="H38" s="135"/>
+    </row>
+    <row r="39" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A39" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="130"/>
-      <c r="C39" s="130"/>
-      <c r="D39" s="130"/>
-      <c r="E39" s="130"/>
-      <c r="F39" s="130"/>
-      <c r="G39" s="129" t="s">
+      <c r="B39" s="64"/>
+      <c r="C39" s="64"/>
+      <c r="D39" s="64"/>
+      <c r="E39" s="64"/>
+      <c r="F39" s="64"/>
+      <c r="G39" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="H39" s="131"/>
-    </row>
-    <row r="40" ht="25" customHeight="1" spans="1:8">
-      <c r="A40" s="132"/>
-      <c r="B40" s="133"/>
-      <c r="C40" s="133"/>
-      <c r="D40" s="133"/>
-      <c r="E40" s="133"/>
-      <c r="F40" s="133"/>
-      <c r="G40" s="134" t="s">
+      <c r="H39" s="65"/>
+    </row>
+    <row r="40" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A40" s="66"/>
+      <c r="B40" s="67"/>
+      <c r="C40" s="67"/>
+      <c r="D40" s="67"/>
+      <c r="E40" s="67"/>
+      <c r="F40" s="67"/>
+      <c r="G40" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="H40" s="135"/>
-    </row>
-    <row r="41" ht="25" customHeight="1" spans="1:8">
-      <c r="A41" s="136"/>
-      <c r="B41" s="137"/>
-      <c r="C41" s="138"/>
-      <c r="D41" s="137"/>
-      <c r="E41" s="139"/>
-      <c r="F41" s="137"/>
-      <c r="G41" s="140" t="s">
+      <c r="H40" s="69"/>
+    </row>
+    <row r="41" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A41" s="70"/>
+      <c r="B41" s="71"/>
+      <c r="C41" s="72"/>
+      <c r="D41" s="71"/>
+      <c r="E41" s="73"/>
+      <c r="F41" s="71"/>
+      <c r="G41" s="74" t="s">
         <v>40</v>
       </c>
-      <c r="H41" s="138"/>
-    </row>
-    <row r="42" ht="25" customHeight="1" spans="1:8">
-      <c r="A42" s="141"/>
-      <c r="B42" s="58"/>
-      <c r="C42" s="142"/>
-      <c r="D42" s="58"/>
-      <c r="E42" s="58"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="143" t="s">
+      <c r="H41" s="72"/>
+    </row>
+    <row r="42" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A42" s="75"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="76"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="H42" s="142"/>
-    </row>
-    <row r="43" ht="25" customHeight="1" spans="1:8">
-      <c r="A43" s="141"/>
-      <c r="B43" s="58"/>
-      <c r="C43" s="142"/>
-      <c r="D43" s="58"/>
-      <c r="E43" s="58"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="144"/>
-      <c r="H43" s="142"/>
-    </row>
-    <row r="44" ht="25" customHeight="1" spans="1:8">
-      <c r="A44" s="141"/>
-      <c r="B44" s="58"/>
-      <c r="C44" s="142"/>
-      <c r="D44" s="58"/>
-      <c r="E44" s="58"/>
-      <c r="F44" s="23"/>
-      <c r="G44" s="144" t="s">
+      <c r="H42" s="76"/>
+    </row>
+    <row r="43" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A43" s="75"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="76"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="78"/>
+      <c r="H43" s="76"/>
+    </row>
+    <row r="44" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A44" s="75"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="76"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="78" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="142"/>
-    </row>
-    <row r="45" ht="25" customHeight="1" spans="1:8">
-      <c r="A45" s="141"/>
-      <c r="B45" s="58"/>
-      <c r="C45" s="142"/>
-      <c r="D45" s="58"/>
-      <c r="E45" s="145"/>
-      <c r="F45" s="23"/>
-      <c r="G45" s="143" t="s">
+      <c r="H44" s="76"/>
+    </row>
+    <row r="45" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A45" s="75"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="76"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="77" t="s">
         <v>43</v>
       </c>
-      <c r="H45" s="142"/>
-    </row>
-    <row r="46" ht="25" customHeight="1" spans="1:8">
-      <c r="A46" s="141"/>
-      <c r="B46" s="58"/>
-      <c r="C46" s="142"/>
-      <c r="D46" s="58"/>
-      <c r="E46" s="100"/>
-      <c r="F46" s="23"/>
-      <c r="G46" s="144"/>
-      <c r="H46" s="142"/>
-    </row>
-    <row r="47" ht="25" customHeight="1" spans="1:8">
-      <c r="A47" s="141"/>
-      <c r="B47" s="58"/>
-      <c r="C47" s="142"/>
-      <c r="D47" s="58"/>
-      <c r="E47" s="100"/>
-      <c r="F47" s="23"/>
-      <c r="G47" s="144" t="s">
+      <c r="H45" s="76"/>
+    </row>
+    <row r="46" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A46" s="75"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="76"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="62"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="78"/>
+      <c r="H46" s="76"/>
+    </row>
+    <row r="47" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A47" s="75"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="76"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="62"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="78" t="s">
         <v>44</v>
       </c>
-      <c r="H47" s="142"/>
-    </row>
-    <row r="48" ht="25" customHeight="1" spans="1:8">
-      <c r="A48" s="141"/>
-      <c r="B48" s="58"/>
-      <c r="C48" s="142"/>
-      <c r="D48" s="58"/>
-      <c r="E48" s="100"/>
-      <c r="F48" s="23"/>
-      <c r="G48" s="146"/>
-      <c r="H48" s="142"/>
-    </row>
-    <row r="49" ht="25" customHeight="1" spans="1:8">
-      <c r="A49" s="141"/>
-      <c r="B49" s="58"/>
-      <c r="C49" s="142"/>
-      <c r="D49" s="58"/>
-      <c r="E49" s="100"/>
-      <c r="F49" s="23"/>
-      <c r="G49" s="144"/>
-      <c r="H49" s="142"/>
-    </row>
-    <row r="50" ht="25" customHeight="1" spans="1:8">
-      <c r="A50" s="141"/>
-      <c r="B50" s="58"/>
-      <c r="C50" s="142"/>
-      <c r="D50" s="58"/>
-      <c r="E50" s="100"/>
-      <c r="F50" s="23"/>
-      <c r="G50" s="141"/>
-      <c r="H50" s="142"/>
-    </row>
-    <row r="51" ht="25" customHeight="1" spans="1:8">
-      <c r="A51" s="141"/>
-      <c r="B51" s="58"/>
-      <c r="C51" s="147"/>
-      <c r="D51" s="58"/>
-      <c r="F51" s="23"/>
-      <c r="G51" s="141"/>
-      <c r="H51" s="142"/>
-    </row>
-    <row r="52" ht="25" customHeight="1" spans="1:8">
-      <c r="A52" s="148"/>
-      <c r="C52" s="149"/>
-      <c r="D52" s="58"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="141"/>
-      <c r="H52" s="142"/>
-    </row>
-    <row r="53" ht="25" customHeight="1" spans="1:8">
-      <c r="A53" s="150" t="s">
+      <c r="H47" s="76"/>
+    </row>
+    <row r="48" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A48" s="75"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="76"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="14"/>
+      <c r="G48" s="79"/>
+      <c r="H48" s="76"/>
+    </row>
+    <row r="49" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A49" s="75"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="76"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="78"/>
+      <c r="H49" s="76"/>
+    </row>
+    <row r="50" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A50" s="75"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="76"/>
+      <c r="D50" s="14"/>
+      <c r="E50" s="62"/>
+      <c r="F50" s="14"/>
+      <c r="G50" s="75"/>
+      <c r="H50" s="76"/>
+    </row>
+    <row r="51" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A51" s="75"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="80"/>
+      <c r="D51" s="14"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="75"/>
+      <c r="H51" s="76"/>
+    </row>
+    <row r="52" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A52" s="81"/>
+      <c r="C52" s="82"/>
+      <c r="D52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="75"/>
+      <c r="H52" s="76"/>
+    </row>
+    <row r="53" spans="1:8" ht="24.95" customHeight="1">
+      <c r="A53" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="B53" s="151"/>
-      <c r="C53" s="152"/>
-      <c r="D53" s="153"/>
-      <c r="E53" s="154"/>
-      <c r="F53" s="153"/>
-      <c r="G53" s="155"/>
-      <c r="H53" s="156"/>
+      <c r="B53" s="101"/>
+      <c r="C53" s="102"/>
+      <c r="D53" s="83"/>
+      <c r="E53" s="84"/>
+      <c r="F53" s="83"/>
+      <c r="G53" s="85"/>
+      <c r="H53" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="G30:H37"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B21:C22"/>
+    <mergeCell ref="A30:B37"/>
+    <mergeCell ref="C30:D37"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="A29:H29"/>
@@ -4448,24 +3918,17 @@
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="G38:H38"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="E30:F37"/>
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="E8:E9"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="B17:C18"/>
-    <mergeCell ref="B21:C22"/>
-    <mergeCell ref="A30:B37"/>
-    <mergeCell ref="C30:D37"/>
-    <mergeCell ref="E30:F37"/>
-    <mergeCell ref="G30:H37"/>
+    <mergeCell ref="F17:G17"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-  <drawing r:id="rId1"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.11811023622047245" bottom="0.11811023622047245" header="0.11811023622047245" footer="0.11811023622047245"/>
+  <pageSetup paperSize="9" scale="36" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>